<commit_message>
chore: update dataset 2026-05-18 and switch map colormap to DENV
- Append DGHS bulletin 2026-05-18: 54,911 suspected, 7,856 confirmed,
  389 suspected deaths, 75 confirmed deaths, 42,868 hospitalised
- Rebuild consolidated Excel dataset
- Replace YlOrRd with cyan→blue→green→red (DENV) colormap on
  division choropleth maps (fig01–fig03); scale bar and compass unchanged
- Regenerate all 18 figures and notebook outputs

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/processed/measles_bangladesh_consolidated.xlsx
+++ b/data/processed/measles_bangladesh_consolidated.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="cases_full" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="mcv1_coverage" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="mcv2_coverage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="outbreak_2026_summary" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="outbreak_2026_divisions" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="outbreak_2026_districts" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="outbreak_2026_timeseries" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="update_log" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cases_full" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="mcv1_coverage" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="mcv2_coverage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="outbreak_2026_summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="outbreak_2026_divisions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="outbreak_2026_districts" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="outbreak_2026_timeseries" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="update_log" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,13 +24,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -51,7 +54,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -59,13 +62,22 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -442,17 +454,17 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Reported_Cases_WHO</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
@@ -890,27 +902,27 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>MCV1_WHO_OrigSource</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>MCV1_Official_%</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>MCV1_Admin_%</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>MCV1_WHO_GHO_%</t>
         </is>
@@ -1368,27 +1380,27 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>MCV2_WHO_OrigSource</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>MCV2_Official_%</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>MCV2_Admin_%</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>MCV2_WHO_GHO_%</t>
         </is>
@@ -1633,12 +1645,12 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -1664,7 +1676,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-18</t>
         </is>
       </c>
     </row>
@@ -1675,7 +1687,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>37131</v>
+        <v>54911</v>
       </c>
     </row>
     <row r="5">
@@ -1685,7 +1697,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5028</v>
+        <v>7856</v>
       </c>
     </row>
     <row r="6">
@@ -1695,7 +1707,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6883</v>
+        <v>42868</v>
       </c>
     </row>
     <row r="7">
@@ -1705,7 +1717,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>227</v>
+        <v>389</v>
       </c>
     </row>
     <row r="8">
@@ -1715,7 +1727,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>49</v>
+        <v>75</v>
       </c>
     </row>
     <row r="9">
@@ -1725,7 +1737,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>276</v>
+        <v>464</v>
       </c>
     </row>
     <row r="10">
@@ -1735,7 +1747,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.74</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="11">
@@ -1796,7 +1808,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>BSS News 2026-04-30 (auto)</t>
+          <t>DGHS daily bulletin 2026-05-18</t>
         </is>
       </c>
     </row>
@@ -1823,32 +1835,32 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Division</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Districts_affected</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Cases</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Deaths</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Pct_of_total</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>CFR_pct</t>
         </is>
@@ -2053,32 +2065,32 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Division</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>District</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Cases</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Deaths</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Pct_of_total</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>CFR_pct</t>
         </is>
@@ -2519,12 +2531,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Dhaka</t>
+          <t>Rajshahi</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Manikgang</t>
+          <t>Pabna</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2543,12 +2555,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Rajshahi</t>
+          <t>Dhaka</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Pabna</t>
+          <t>Manikgang</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2735,49 +2747,49 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Chattogram</t>
+          <t>Rangpur</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Coxsbazar</t>
+          <t>Thakurgaon</t>
         </is>
       </c>
       <c r="C29" t="n">
         <v>31</v>
       </c>
       <c r="D29" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E29" t="n">
         <v>0.27</v>
       </c>
       <c r="F29" t="n">
-        <v>16.13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Rangpur</t>
+          <t>Chattogram</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Thakurgaon</t>
+          <t>Coxsbazar</t>
         </is>
       </c>
       <c r="C30" t="n">
         <v>31</v>
       </c>
       <c r="D30" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E30" t="n">
         <v>0.27</v>
       </c>
       <c r="F30" t="n">
-        <v>0</v>
+        <v>16.13</v>
       </c>
     </row>
     <row r="31">
@@ -2831,12 +2843,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Mymensingh</t>
+          <t>Khulna</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Sherpur</t>
+          <t>Norail</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -2879,12 +2891,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Khulna</t>
+          <t>Mymensingh</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Norail</t>
+          <t>Sherpur</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -2999,12 +3011,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Dhaka</t>
+          <t>Khulna</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Narshindi</t>
+          <t>Jhinadah</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -3023,12 +3035,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Khulna</t>
+          <t>Dhaka</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Jhinadah</t>
+          <t>Narshindi</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -3143,12 +3155,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Rangpur</t>
+          <t>Barisal</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Gaibanda</t>
+          <t>Pirozpur</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -3167,12 +3179,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Barisal</t>
+          <t>Rangpur</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Pirozpur</t>
+          <t>Gaibanda</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -3407,49 +3419,49 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Rajshahi</t>
+          <t>Rangpur</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Naogan</t>
+          <t>Dinajpur</t>
         </is>
       </c>
       <c r="C57" t="n">
         <v>2</v>
       </c>
       <c r="D57" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E57" t="n">
         <v>0.02</v>
       </c>
       <c r="F57" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Rangpur</t>
+          <t>Rajshahi</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Dinajpur</t>
+          <t>Naogan</t>
         </is>
       </c>
       <c r="C58" t="n">
         <v>2</v>
       </c>
       <c r="D58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E58" t="n">
         <v>0.02</v>
       </c>
       <c r="F58" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="59">
@@ -3535,7 +3547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3551,52 +3563,52 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Suspected_Cases</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Confirmed_Cases</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Hospitalised</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Suspected_Deaths</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Confirmed_Deaths</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Districts_Affected</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Total_Deaths</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>CFR_pct</t>
         </is>
@@ -3795,6 +3807,39 @@
       </c>
       <c r="J7" t="n">
         <v>0.74</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>54911</v>
+      </c>
+      <c r="C8" t="n">
+        <v>7856</v>
+      </c>
+      <c r="D8" t="n">
+        <v>42868</v>
+      </c>
+      <c r="E8" t="n">
+        <v>389</v>
+      </c>
+      <c r="F8" t="n">
+        <v>75</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>DGHS daily bulletin 2026-05-18</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>464</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.85</v>
       </c>
     </row>
   </sheetData>
@@ -3822,42 +3867,42 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Updated</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Source_Cases</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Source_MCV1</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Source_MCV2</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Source_2026</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Cases_rows</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>MCV1_rows</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>MCV2_rows</t>
         </is>
@@ -3866,7 +3911,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-18T08:36:50</t>
+          <t>2026-05-18T16:58:48</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>